<commit_message>
Receipt benchmark Phase 1: verified ground truth and multi-approach scoring
- Ground truth: r3 doctor Becku -> Becky and r2 patient na -> Carol Tse (both
  checked against the receipt images); dates stored as ISO text instead of
  Excel serials. Open questions logged in GROUND_TRUTH_REVIEW.md.
- score.py: score any number of named approaches (--approach NAME=DIR) on the
  six fields as Correct / Wrong / N/A. Accuracy = correct / applicable; invented
  values on N/A fields reported separately; failed runs and missing results
  count as wrong; no day/month swapping; visit_date -> service_date alias.
  Writes report.md, summary.csv and detail.csv.
- Tests for ground-truth loading, normalization, marking, field mapping and
  scoring four approaches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/python/receipt_ocr_benchmark/data/ground_truth/ground_truth_template.xlsx
+++ b/python/receipt_ocr_benchmark/data/ground_truth/ground_truth_template.xlsx
@@ -77,7 +77,7 @@
     <t>na</t>
   </si>
   <si>
-    <t>Lee Tin Tin, Becku</t>
+    <t>Lee Tin Tin, Becky</t>
   </si>
   <si>
     <t>Angel Tseng, Lok Yi Choi</t>
@@ -497,8 +497,10 @@
       <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="1">
-        <v>46205</v>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
       </c>
       <c r="G2" s="1">
         <v>1540</v>
@@ -514,14 +516,18 @@
       <c r="C3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>17</v>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Carol Tse</t>
+        </is>
       </c>
       <c r="E3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1">
-        <v>46333</v>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
       </c>
       <c r="G3" s="1">
         <v>998</v>
@@ -543,8 +549,10 @@
       <c r="E4" s="1">
         <v>967157032</v>
       </c>
-      <c r="F4" s="1">
-        <v>46204</v>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
       </c>
       <c r="G4" s="1">
         <v>10</v>
@@ -566,8 +574,10 @@
       <c r="E5" s="1">
         <v>369303</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>21</v>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>2023-02-09</t>
+        </is>
       </c>
       <c r="G5" s="1">
         <v>1361</v>
@@ -589,8 +599,10 @@
       <c r="E6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="1">
-        <v>46266</v>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
       </c>
       <c r="G6" s="1">
         <v>20</v>
@@ -612,8 +624,10 @@
       <c r="E7" s="1">
         <v>9990000505906</v>
       </c>
-      <c r="F7" s="1">
-        <v>42818</v>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>2017-03-24</t>
+        </is>
       </c>
       <c r="G7" s="1">
         <v>51.2</v>

</xml_diff>